<commit_message>
refactor: v3.1 code cleanup & version standardization
- Created src/utils/helpers.py: centralized shared utilities (save_leads_to_file, extract_emails_from_website, parse_lead_name)
- Refactored src/gui/dentist_lead_suite_gui.py: removed duplicate helper functions (~70 lines), standardized fallback imports, updated all headers & status bars to v3.1
- Refactored src/scraper/free_dentist_scraper.py: imported helpers, integrated system optimizer & per-city dedup registry into CLI mode
- Standardized version strings to v3.1 across main.py, categories.py, README.md, docs/HOW_TO_USE.md
</commit_message>
<xml_diff>
--- a/output/Dentists_Ahmedabad_Leads.xlsx
+++ b/output/Dentists_Ahmedabad_Leads.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aayus\Desktop\Dentist-Lead-Scraper-Suite\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D2DF00F-D19C-40F0-87F2-FDBAED8A633F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93F5B0C8-73AA-4CE1-AD64-505095C53241}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="86">
   <si>
     <t>City</t>
   </si>
@@ -72,214 +72,217 @@
     <t>Ahmedabad</t>
   </si>
   <si>
-    <t>Maninagar</t>
+    <t>Satellite</t>
   </si>
   <si>
     <t>🦷 Dentists</t>
   </si>
   <si>
+    <t>Dhwanil</t>
+  </si>
+  <si>
+    <t>Dental</t>
+  </si>
+  <si>
+    <t>Dhwanil Dental Clinic</t>
+  </si>
+  <si>
+    <t>098794 06548</t>
+  </si>
+  <si>
+    <t>Jodhpur Gam Rd, Satellite, Ahmedabad, Gujarat 380015</t>
+  </si>
+  <si>
+    <t>4.9 ★</t>
+  </si>
+  <si>
+    <t>448</t>
+  </si>
+  <si>
+    <t>http://dhwanildental.com/</t>
+  </si>
+  <si>
+    <t>info.dhwanildentalclinic@gmail.com</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/place/Dhwanil+Dental+Clinic/data=!4m7!3m6!1s0x395e84cdf0ce25ad:0xaafdde7b37945037!8m2!3d23.0217318!4d72.5253185!16s%2Fg%2F1264gw8yd!19sChIJrSXO8M2EXjkRN1CUN3ve_ao</t>
+  </si>
+  <si>
+    <t>Agrawals</t>
+  </si>
+  <si>
+    <t>Multi</t>
+  </si>
+  <si>
+    <t>Agrawal's Multi Speciality Dental Clinic</t>
+  </si>
+  <si>
+    <t>079 2673 0229</t>
+  </si>
+  <si>
+    <t>B, 105, Shital Varsha Complex, 104, Shivranjani Cross Rd, near Kalupur Commercial Bank, Suryapooja Block B, Satellite, Ahmedabad, Gujarat 380015</t>
+  </si>
+  <si>
+    <t>5.0 ★</t>
+  </si>
+  <si>
+    <t>813</t>
+  </si>
+  <si>
+    <t>https://agrawaldentalclinic.com/</t>
+  </si>
+  <si>
+    <t>No Email Found</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/place/Agrawal%27s+Multi+Speciality+Dental+Clinic/data=!4m7!3m6!1s0x395e84cfb7081ff5:0x846a653dcfa4202b!8m2!3d23.0247942!4d72.5294606!16s%2Fg%2F1pp2tzrc4!19sChIJ9R8It8-EXjkRKyCkzz1laoQ</t>
+  </si>
+  <si>
+    <t>Shree</t>
+  </si>
+  <si>
+    <t>Shree Dental Care</t>
+  </si>
+  <si>
+    <t>098252 58149</t>
+  </si>
+  <si>
+    <t>Second Floor, Goldcoin Complex, 3B, Jodhpur Cross Rd, Kameshwar Vihar, Suryapooja Block B, Satellite, Ahmedabad, Gujarat 380015</t>
+  </si>
+  <si>
+    <t>140</t>
+  </si>
+  <si>
+    <t>http://shreedentalcare.com/</t>
+  </si>
+  <si>
+    <t>drjayshreeraiya@yahoo.co.in</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/place/Shree+Dental+Care/data=!4m7!3m6!1s0x395e84b62e55cb9f:0xec2e87982ffa2dbd!8m2!3d23.0259005!4d72.5273727!16s%2Fg%2F1vg_b7zx!19sChIJn8tVLraEXjkRvS36L5iHLuw</t>
+  </si>
+  <si>
+    <t>Teeth</t>
+  </si>
+  <si>
+    <t>Care</t>
+  </si>
+  <si>
+    <t>Teeth Care Centre® Dental Hospital [High-end Dentistry]</t>
+  </si>
+  <si>
+    <t>No Phone Listed</t>
+  </si>
+  <si>
+    <t>2nd Floor, Pushpak66, 132 Feet Ring Rd, near Someshwar Jain Temple, Satellite, Ahmedabad, Gujarat 380015</t>
+  </si>
+  <si>
+    <t>6,277</t>
+  </si>
+  <si>
+    <t>https://www.teethcarecentre.com/</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/place/Teeth+Care+Centre%C2%AE+Dental+Hospital+%5BHigh-end+Dentistry%5D/data=!4m7!3m6!1s0x395e84d0da686b69:0x8ed8388cff8ab64e!8m2!3d23.0180608!4d72.5299026!16s%2Fg%2F1vyk0xlc!19sChIJaWto2tCEXjkRTraK_4w42I4</t>
+  </si>
+  <si>
+    <t>Sabka</t>
+  </si>
+  <si>
     <t>Dentist</t>
   </si>
   <si>
-    <t>Kanishka</t>
-  </si>
-  <si>
-    <t>Dentist Kanishka Dental Clinic</t>
-  </si>
-  <si>
-    <t>098796 09227</t>
-  </si>
-  <si>
-    <t>Bhadwatnagar, Ghodasar,maninagar Opp.yamunaji haveli , opp.shlok hospital ,nr .jaymala,isanpur, road, Maninagar, Ahmedabad, Gujarat 380008</t>
-  </si>
-  <si>
-    <t>5.0 ★</t>
-  </si>
-  <si>
-    <t>69</t>
-  </si>
-  <si>
-    <t>No Website</t>
-  </si>
-  <si>
-    <t>No Email Found</t>
-  </si>
-  <si>
-    <t>No</t>
-  </si>
-  <si>
-    <t>https://www.google.com/maps/place/Dentist+Kanishka+Dental+Clinic/data=!4m7!3m6!1s0x395e85997d60b527:0x9448585e2eab5085!8m2!3d22.9872466!4d72.603168!16s%2Fg%2F11f5q0bs2_!19sChIJJ7VgfZmFXjkRhVCrLl5YSJQ</t>
-  </si>
-  <si>
-    <t>Dr</t>
-  </si>
-  <si>
-    <t>Mehtas</t>
-  </si>
-  <si>
-    <t>Dr Mehta's Dental Care</t>
-  </si>
-  <si>
-    <t>094285 63659</t>
-  </si>
-  <si>
-    <t>C/106 Janpath Society Ghodasar Canal Garden, Road, near aavkar hall, Maninagar, Ahmedabad, Gujarat 380050</t>
-  </si>
-  <si>
-    <t>692</t>
-  </si>
-  <si>
-    <t>https://www.drmehtasdentalcare.com/</t>
-  </si>
-  <si>
-    <t>https://www.google.com/maps/place/Dr+Mehta%27s+Dental+Care/data=!4m7!3m6!1s0x395e85e4956c0a29:0xcd077d9ed27b57b9!8m2!3d22.9874219!4d72.6078495!16s%2Fg%2F11gflt43xl!19sChIJKQpsleSFXjkRuVd70p59B80</t>
-  </si>
-  <si>
-    <t>Shahs</t>
-  </si>
-  <si>
-    <t>Dr. Shah's Dental Clinic and Implant Center</t>
-  </si>
-  <si>
-    <t>098984 59197</t>
-  </si>
-  <si>
-    <t>A, A/304, RADHE KISHAN VILLA, near Ratan Hospital, Jaymala, Maninagar, Ahmedabad, Gujarat 380008</t>
-  </si>
-  <si>
-    <t>157</t>
-  </si>
-  <si>
-    <t>https://drchitrangshah.com/</t>
-  </si>
-  <si>
-    <t>https://www.google.com/maps/place/Dr.+Shah%27s+Dental+Clinic+and+Implant+Center/data=!4m7!3m6!1s0x395e81bc4706d3a7:0xfbb83b509bba9740!8m2!3d22.9836515!4d72.6002664!16s%2Fg%2F11h0v8srzh!19sChIJp9MGR7yBXjkRQJe6m1A7uPs</t>
-  </si>
-  <si>
-    <t>Dental</t>
-  </si>
-  <si>
-    <t>Maninagar Dental Hospital &amp; Implant Center</t>
-  </si>
-  <si>
-    <t>085304 50250</t>
-  </si>
-  <si>
-    <t>1st Floor, Sidhpura Complex, opp. Vijay sales, Krishna Baug, Maninagar, Ahmedabad, Gujarat 380008</t>
-  </si>
-  <si>
-    <t>326</t>
-  </si>
-  <si>
-    <t>https://maninagardental.com/</t>
-  </si>
-  <si>
-    <t>https://www.google.com/maps/place/Maninagar+Dental+Hospital+%26+Implant+Center/data=!4m7!3m6!1s0x395e859d7f7a9ba7:0x64f89b96be3e71bb!8m2!3d22.9974727!4d72.6050686!16s%2Fg%2F11hds4bxk1!19sChIJp5t6f52FXjkRu3E-vpab-GQ</t>
-  </si>
-  <si>
-    <t>Shah</t>
-  </si>
-  <si>
-    <t>SHAH DENTAL CLINIC</t>
-  </si>
-  <si>
-    <t>090164 47332</t>
-  </si>
-  <si>
-    <t>Ff/7, Krishna Avenue, BRTS Stand, Gopal Chowk Cross Road, Bhairavnath Rd, Rambagh, Maninagar, Ahmedabad, Gujarat 380008</t>
-  </si>
-  <si>
-    <t>4.9 ★</t>
-  </si>
-  <si>
-    <t>1,235</t>
-  </si>
-  <si>
-    <t>http://www.shahdentalclinic.co.in/</t>
-  </si>
-  <si>
-    <t>shahdentalclinicabd@gmail.com</t>
-  </si>
-  <si>
-    <t>https://www.google.com/maps/place/SHAH+DENTAL+CLINIC/data=!4m7!3m6!1s0x395e8513ed73e017:0x6a7b7968780618f4!8m2!3d22.995554!4d72.5997684!16s%2Fg%2F11f62rwmj_!19sChIJF-Bz7ROFXjkR9BgGeGh5e2o</t>
-  </si>
-  <si>
-    <t>O</t>
-  </si>
-  <si>
-    <t>Shreeji</t>
-  </si>
-  <si>
-    <t>O Shreeji Dental Clinic And Implant Centre</t>
-  </si>
-  <si>
-    <t>094268 63675</t>
-  </si>
-  <si>
-    <t>E/2, Ishwarnagar Society, near TOWER-2, Uttamnagar, Maninagar, Ahmedabad, Gujarat 380008</t>
+    <t>Sabka dentist</t>
+  </si>
+  <si>
+    <t>090811 06611</t>
+  </si>
+  <si>
+    <t>Shyamal Row Houses, Shop No 18, F F Dhananjay Tower, B/H 3/B, 100 Fort Ring Road, Satellite, Ahmedabad, Gujarat 380015</t>
+  </si>
+  <si>
+    <t>4.6 ★</t>
+  </si>
+  <si>
+    <t>1,492</t>
+  </si>
+  <si>
+    <t>https://www.sabkadentist.com/dental-clinics-in-ahmedabad/satellite/</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/place/Sabka+dentist/data=!4m7!3m6!1s0x395e84da52a4944b:0x37d988fae6412707!8m2!3d23.0133945!4d72.5254499!16s%2Fg%2F11b67m922x!19sChIJS5SkUtqEXjkRBydB5vqI2Tc</t>
+  </si>
+  <si>
+    <t>Gmdc</t>
+  </si>
+  <si>
+    <t>GMDC Dental Clinic - Satellite</t>
+  </si>
+  <si>
+    <t>091044 12349</t>
+  </si>
+  <si>
+    <t>Third floor, Goldcoin Complex, B-04, Jodhpur Cross Rd, Kameshwar Vihar, Suryapooja Block B, Satellite, Ahmedabad, Gujarat 380015</t>
+  </si>
+  <si>
+    <t>171</t>
+  </si>
+  <si>
+    <t>https://gmdcdental.com/</t>
+  </si>
+  <si>
+    <t>gmdcdentalclinic@gmail.com</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/place/GMDC+Dental+Clinic+-+Satellite/data=!4m7!3m6!1s0x395e852e1484a795:0x972210a68be5180a!8m2!3d23.0256643!4d72.5270547!16s%2Fg%2F11md2wgzrm!19sChIJlaeEFC6FXjkRChjli6YQIpc</t>
+  </si>
+  <si>
+    <t>Ivories</t>
+  </si>
+  <si>
+    <t>IVORIES DENTAL</t>
+  </si>
+  <si>
+    <t>098983 04506</t>
+  </si>
+  <si>
+    <t>303,304, Maulik Arcade, 302, Judges Bunglow Rd, opp. MANSI TOWER, above KARNAVATI PAGARKHA BAZAAR, JAYMA SOCIETY, Vastrapur, Ahmedabad, Gujarat 380015</t>
   </si>
   <si>
     <t>4.8 ★</t>
   </si>
   <si>
-    <t>64</t>
-  </si>
-  <si>
-    <t>http://www.dentalimplantindia.com/</t>
-  </si>
-  <si>
-    <t>oshreeji.dent@gmail.com</t>
-  </si>
-  <si>
-    <t>https://www.google.com/maps/place/O+Shreeji+Dental+Clinic+And+Implant+Centre/data=!4m7!3m6!1s0x395e848ac8a7faf3:0xf148133acab3e2a4!8m2!3d22.9889072!4d72.6035904!16s%2Fg%2F1td9ny6p!19sChIJ8_qnyIqEXjkRpOKzyjoTSPE</t>
-  </si>
-  <si>
-    <t>World</t>
-  </si>
-  <si>
-    <t>Dental World</t>
-  </si>
-  <si>
-    <t>099099 27737</t>
-  </si>
-  <si>
-    <t>101/ rushabhraj avenue, Isanpur Rd, near vashisthnagar busstand, Maninagar, Ahmedabad, Gujarat 380008</t>
-  </si>
-  <si>
-    <t>17</t>
-  </si>
-  <si>
-    <t>https://drdeeppandya.getmy.clinic/?utm_source=gmb&amp;utm_medium=web&amp;utm_campaign=tu</t>
-  </si>
-  <si>
-    <t>gayatri.behal@remedoapp.com</t>
-  </si>
-  <si>
-    <t>https://www.google.com/maps/place/Dental+World/data=!4m7!3m6!1s0x395e85eff210689b:0x5f0dbeb0b0f1c0b2!8m2!3d22.986516!4d72.6025628!16s%2Fg%2F11f_j3v7zn!19sChIJm2gQ8u-FXjkRssDxsLC-DV8</t>
-  </si>
-  <si>
-    <t>Shrey</t>
-  </si>
-  <si>
-    <t>Shrey Dental Clinic</t>
-  </si>
-  <si>
-    <t>098981 12113</t>
-  </si>
-  <si>
-    <t>Takshashila Square, 301-303, Nirant Cross Rd, opposite Sankalp Restaurant, Krishna Baug, Bhagyanagar Society, Maninagar, Ahmedabad, Gujarat 380008</t>
-  </si>
-  <si>
-    <t>666</t>
-  </si>
-  <si>
-    <t>https://shreydentalclinic.com/</t>
-  </si>
-  <si>
-    <t>shreydentalclinic@gmail.com</t>
-  </si>
-  <si>
-    <t>https://www.google.com/maps/place/Shrey+Dental+Clinic/data=!4m7!3m6!1s0x395e85e7f1291295:0x2ff2bb2fd83d5121!8m2!3d22.9968169!4d72.6039478!16s%2Fg%2F1tk_mp6h!19sChIJlRIp8eeFXjkRIVE92C-78i8</t>
+    <t>1,250</t>
+  </si>
+  <si>
+    <t>http://www.ivoriesdentalclinic.com/</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/place/IVORIES+DENTAL/data=!4m7!3m6!1s0x395e84cbd14722af:0xb33c32c330c90c63!8m2!3d23.0310288!4d72.5261369!16s%2Fg%2F1q6kk5prs!19sChIJryJH0cuEXjkRYwzJMMMyPLM</t>
+  </si>
+  <si>
+    <t>Shwet</t>
+  </si>
+  <si>
+    <t>SHWET DENTAL CLINIC</t>
+  </si>
+  <si>
+    <t>098987 44107</t>
+  </si>
+  <si>
+    <t>F/8, First Floor, Satyam Nr. Prernatirth Derasar, Jodhpur, Satellite, Ahmedabad, Gujarat 380015</t>
+  </si>
+  <si>
+    <t>765</t>
+  </si>
+  <si>
+    <t>http://www.shwetdental.com/</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/place/SHWET+DENTAL+CLINIC/data=!4m7!3m6!1s0x395e9b2ce3a51a31:0x1b866c79ea78873a!8m2!3d23.0189725!4d72.5187339!16s%2Fg%2F1xg5r1_x!19sChIJMRql4yybXjkROod46nlshhs</t>
   </si>
 </sst>
 </file>
@@ -620,22 +623,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:N9"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.5546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.77734375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9.77734375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="8.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="37.5546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.77734375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="126.77734375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="47.44140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="139.109375" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="6.109375" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="79.21875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="27.6640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="59.5546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="31.109375" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="210.6640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="227" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.3">
@@ -752,22 +755,22 @@
         <v>32</v>
       </c>
       <c r="I3" t="s">
-        <v>22</v>
+        <v>33</v>
       </c>
       <c r="J3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="K3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="L3" t="s">
-        <v>25</v>
+        <v>36</v>
       </c>
       <c r="M3" t="s">
         <v>26</v>
       </c>
       <c r="N3" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.3">
@@ -781,37 +784,37 @@
         <v>16</v>
       </c>
       <c r="D4" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="E4" t="s">
-        <v>36</v>
+        <v>18</v>
       </c>
       <c r="F4" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="G4" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="H4" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="I4" t="s">
         <v>22</v>
       </c>
       <c r="J4" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="K4" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="L4" t="s">
-        <v>25</v>
+        <v>44</v>
       </c>
       <c r="M4" t="s">
         <v>26</v>
       </c>
       <c r="N4" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.3">
@@ -825,37 +828,37 @@
         <v>16</v>
       </c>
       <c r="D5" t="s">
-        <v>15</v>
+        <v>46</v>
       </c>
       <c r="E5" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="F5" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="G5" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="H5" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="I5" t="s">
-        <v>22</v>
+        <v>33</v>
       </c>
       <c r="J5" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="K5" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="L5" t="s">
-        <v>25</v>
+        <v>36</v>
       </c>
       <c r="M5" t="s">
         <v>26</v>
       </c>
       <c r="N5" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.3">
@@ -869,37 +872,37 @@
         <v>16</v>
       </c>
       <c r="D6" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="E6" t="s">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="F6" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="G6" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="H6" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="I6" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="J6" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="K6" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="L6" t="s">
-        <v>57</v>
+        <v>36</v>
       </c>
       <c r="M6" t="s">
         <v>26</v>
       </c>
       <c r="N6" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
@@ -913,37 +916,37 @@
         <v>16</v>
       </c>
       <c r="D7" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="E7" t="s">
-        <v>60</v>
+        <v>18</v>
       </c>
       <c r="F7" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="G7" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="H7" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="I7" t="s">
-        <v>64</v>
+        <v>33</v>
       </c>
       <c r="J7" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="K7" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="L7" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="M7" t="s">
         <v>26</v>
       </c>
       <c r="N7" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.3">
@@ -957,37 +960,37 @@
         <v>16</v>
       </c>
       <c r="D8" t="s">
-        <v>43</v>
+        <v>71</v>
       </c>
       <c r="E8" t="s">
-        <v>69</v>
+        <v>18</v>
       </c>
       <c r="F8" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G8" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="H8" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="I8" t="s">
-        <v>22</v>
+        <v>75</v>
       </c>
       <c r="J8" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="K8" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="L8" t="s">
-        <v>75</v>
+        <v>36</v>
       </c>
       <c r="M8" t="s">
         <v>26</v>
       </c>
       <c r="N8" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.3">
@@ -1001,37 +1004,37 @@
         <v>16</v>
       </c>
       <c r="D9" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="E9" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="F9" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="G9" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="H9" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="I9" t="s">
-        <v>54</v>
+        <v>33</v>
       </c>
       <c r="J9" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="K9" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="L9" t="s">
-        <v>83</v>
+        <v>36</v>
       </c>
       <c r="M9" t="s">
         <v>26</v>
       </c>
       <c r="N9" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
   </sheetData>

</xml_diff>